<commit_message>
Optimización móvil de evaluador.html y remoción de botón público
</commit_message>
<xml_diff>
--- a/SIG_MotMot_Validacion_Campo.xlsx
+++ b/SIG_MotMot_Validacion_Campo.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="250">
   <si>
     <t>type</t>
   </si>
@@ -259,9 +259,6 @@
   </si>
   <si>
     <t>minimal</t>
-  </si>
-  <si>
-    <t>search</t>
   </si>
   <si>
     <t>new</t>
@@ -1254,9 +1251,6 @@
       <c r="D3" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>81</v>
-      </c>
     </row>
     <row r="4" spans="1:6" ht="20" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -1297,7 +1291,7 @@
         <v>54</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="20" customHeight="1">
@@ -1328,7 +1322,7 @@
         <v>78</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="20" customHeight="1">
@@ -1401,7 +1395,7 @@
         <v>78</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="20" customHeight="1">
@@ -1423,7 +1417,7 @@
         <v>62</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="20" customHeight="1">
@@ -1454,7 +1448,7 @@
         <v>78</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="20" customHeight="1">
@@ -1485,7 +1479,7 @@
         <v>78</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:6" ht="20" customHeight="1">
@@ -1516,7 +1510,7 @@
         <v>78</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="22" spans="1:6" ht="20" customHeight="1">
@@ -1547,7 +1541,7 @@
         <v>79</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="20" customHeight="1">
@@ -1564,7 +1558,7 @@
         <v>78</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:6" ht="20" customHeight="1">
@@ -1586,7 +1580,7 @@
         <v>72</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="20" customHeight="1">
@@ -1617,7 +1611,7 @@
         <v>78</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="29" spans="1:6" ht="20" customHeight="1">
@@ -1670,7 +1664,7 @@
         <v>79</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1688,7 +1682,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="30" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -1702,10 +1696,10 @@
         <v>22</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="20" customHeight="1">
@@ -1713,10 +1707,10 @@
         <v>22</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="20" customHeight="1">
@@ -1724,10 +1718,10 @@
         <v>23</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="20" customHeight="1">
@@ -1735,10 +1729,10 @@
         <v>23</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="20" customHeight="1">
@@ -1746,10 +1740,10 @@
         <v>23</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="20" customHeight="1">
@@ -1757,10 +1751,10 @@
         <v>23</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="20" customHeight="1">
@@ -1768,10 +1762,10 @@
         <v>23</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="20" customHeight="1">
@@ -1779,10 +1773,10 @@
         <v>23</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="20" customHeight="1">
@@ -1790,10 +1784,10 @@
         <v>23</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="20" customHeight="1">
@@ -1801,10 +1795,10 @@
         <v>23</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="20" customHeight="1">
@@ -1812,10 +1806,10 @@
         <v>23</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="20" customHeight="1">
@@ -1823,10 +1817,10 @@
         <v>23</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="20" customHeight="1">
@@ -1834,10 +1828,10 @@
         <v>23</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="20" customHeight="1">
@@ -1845,10 +1839,10 @@
         <v>23</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="20" customHeight="1">
@@ -1856,10 +1850,10 @@
         <v>23</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="20" customHeight="1">
@@ -1867,10 +1861,10 @@
         <v>23</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="20" customHeight="1">
@@ -1878,10 +1872,10 @@
         <v>23</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="20" customHeight="1">
@@ -1889,10 +1883,10 @@
         <v>23</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="20" customHeight="1">
@@ -1900,10 +1894,10 @@
         <v>23</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="20" customHeight="1">
@@ -1911,10 +1905,10 @@
         <v>23</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="20" customHeight="1">
@@ -1922,10 +1916,10 @@
         <v>23</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="20" customHeight="1">
@@ -1933,10 +1927,10 @@
         <v>23</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="20" customHeight="1">
@@ -1944,10 +1938,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="20" customHeight="1">
@@ -1955,10 +1949,10 @@
         <v>23</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="20" customHeight="1">
@@ -1966,10 +1960,10 @@
         <v>23</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="20" customHeight="1">
@@ -1977,10 +1971,10 @@
         <v>23</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="20" customHeight="1">
@@ -1988,10 +1982,10 @@
         <v>23</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="20" customHeight="1">
@@ -1999,10 +1993,10 @@
         <v>24</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="20" customHeight="1">
@@ -2010,10 +2004,10 @@
         <v>24</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="20" customHeight="1">
@@ -2021,10 +2015,10 @@
         <v>24</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="20" customHeight="1">
@@ -2032,10 +2026,10 @@
         <v>24</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="20" customHeight="1">
@@ -2043,10 +2037,10 @@
         <v>24</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="20" customHeight="1">
@@ -2054,10 +2048,10 @@
         <v>24</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="20" customHeight="1">
@@ -2065,10 +2059,10 @@
         <v>27</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="20" customHeight="1">
@@ -2076,10 +2070,10 @@
         <v>27</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="20" customHeight="1">
@@ -2087,10 +2081,10 @@
         <v>27</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="20" customHeight="1">
@@ -2098,10 +2092,10 @@
         <v>27</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="20" customHeight="1">
@@ -2109,10 +2103,10 @@
         <v>27</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="20" customHeight="1">
@@ -2120,10 +2114,10 @@
         <v>27</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="20" customHeight="1">
@@ -2131,10 +2125,10 @@
         <v>30</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="20" customHeight="1">
@@ -2142,10 +2136,10 @@
         <v>30</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="20" customHeight="1">
@@ -2153,10 +2147,10 @@
         <v>30</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="20" customHeight="1">
@@ -2164,10 +2158,10 @@
         <v>30</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="20" customHeight="1">
@@ -2175,10 +2169,10 @@
         <v>31</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="20" customHeight="1">
@@ -2186,10 +2180,10 @@
         <v>31</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="20" customHeight="1">
@@ -2197,10 +2191,10 @@
         <v>31</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="20" customHeight="1">
@@ -2208,10 +2202,10 @@
         <v>31</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="20" customHeight="1">
@@ -2219,307 +2213,307 @@
         <v>31</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="20" customHeight="1">
       <c r="A50" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="20" customHeight="1">
       <c r="A51" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="20" customHeight="1">
       <c r="A52" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="20" customHeight="1">
       <c r="A53" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="20" customHeight="1">
       <c r="A54" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="20" customHeight="1">
       <c r="A55" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="20" customHeight="1">
       <c r="A56" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="20" customHeight="1">
       <c r="A57" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="20" customHeight="1">
       <c r="A58" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="20" customHeight="1">
       <c r="A59" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="20" customHeight="1">
       <c r="A60" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="20" customHeight="1">
       <c r="A61" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="20" customHeight="1">
       <c r="A62" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="20" customHeight="1">
       <c r="A63" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="20" customHeight="1">
       <c r="A64" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="20" customHeight="1">
       <c r="A65" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="20" customHeight="1">
       <c r="A66" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="20" customHeight="1">
       <c r="A67" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="20" customHeight="1">
       <c r="A68" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="20" customHeight="1">
       <c r="A69" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="20" customHeight="1">
       <c r="A70" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="20" customHeight="1">
       <c r="A71" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="20" customHeight="1">
       <c r="A72" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="20" customHeight="1">
       <c r="A73" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="20" customHeight="1">
       <c r="A74" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="20" customHeight="1">
       <c r="A75" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="20" customHeight="1">
       <c r="A76" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
   </sheetData>
@@ -2537,36 +2531,36 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
       <c r="A1" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>244</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>245</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="100" customHeight="1">
       <c r="A2" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>249</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrección responsiva: Ajuste multilínea en botones de interfaz móvil
</commit_message>
<xml_diff>
--- a/SIG_MotMot_Validacion_Campo.xlsx
+++ b/SIG_MotMot_Validacion_Campo.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="252">
   <si>
     <t>type</t>
   </si>
@@ -315,6 +315,9 @@
     <t>antonio</t>
   </si>
   <si>
+    <t>alexander</t>
+  </si>
+  <si>
     <t>w_barichara</t>
   </si>
   <si>
@@ -522,10 +525,13 @@
     <t>patrimonio</t>
   </si>
   <si>
-    <t>Liliana Paola Rozo Martínez</t>
-  </si>
-  <si>
-    <t>Antonio José Becerra Velásquez</t>
+    <t>Liliana Paola Rozo Martínez - Gerente General / Auditora</t>
+  </si>
+  <si>
+    <t>Antonio José Becerra Velásquez - Guía Turístico Profesional</t>
+  </si>
+  <si>
+    <t>Alexander Jimenez - Guía Turístico Profesional</t>
   </si>
   <si>
     <t>Servicio 1: Walking Tour Barichara</t>
@@ -1674,7 +1680,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F77"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="6" width="28.7109375" style="1" customWidth="1"/>
@@ -1699,7 +1705,7 @@
         <v>97</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="20" customHeight="1">
@@ -1710,18 +1716,18 @@
         <v>98</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="20" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>99</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="20" customHeight="1">
@@ -1732,7 +1738,7 @@
         <v>100</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="20" customHeight="1">
@@ -1743,7 +1749,7 @@
         <v>101</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="20" customHeight="1">
@@ -1754,7 +1760,7 @@
         <v>102</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="20" customHeight="1">
@@ -1765,7 +1771,7 @@
         <v>103</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="20" customHeight="1">
@@ -1776,7 +1782,7 @@
         <v>104</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="20" customHeight="1">
@@ -1787,7 +1793,7 @@
         <v>105</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="20" customHeight="1">
@@ -1798,7 +1804,7 @@
         <v>106</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="20" customHeight="1">
@@ -1809,7 +1815,7 @@
         <v>107</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="20" customHeight="1">
@@ -1820,7 +1826,7 @@
         <v>108</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="20" customHeight="1">
@@ -1831,7 +1837,7 @@
         <v>109</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="20" customHeight="1">
@@ -1842,7 +1848,7 @@
         <v>110</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="20" customHeight="1">
@@ -1853,7 +1859,7 @@
         <v>111</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="20" customHeight="1">
@@ -1864,7 +1870,7 @@
         <v>112</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="20" customHeight="1">
@@ -1875,7 +1881,7 @@
         <v>113</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="20" customHeight="1">
@@ -1886,7 +1892,7 @@
         <v>114</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="20" customHeight="1">
@@ -1897,7 +1903,7 @@
         <v>115</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="20" customHeight="1">
@@ -1908,7 +1914,7 @@
         <v>116</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="20" customHeight="1">
@@ -1919,7 +1925,7 @@
         <v>117</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="20" customHeight="1">
@@ -1930,7 +1936,7 @@
         <v>118</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="20" customHeight="1">
@@ -1941,7 +1947,7 @@
         <v>119</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="20" customHeight="1">
@@ -1952,7 +1958,7 @@
         <v>120</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="20" customHeight="1">
@@ -1963,7 +1969,7 @@
         <v>121</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="20" customHeight="1">
@@ -1974,7 +1980,7 @@
         <v>122</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="20" customHeight="1">
@@ -1985,18 +1991,18 @@
         <v>123</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="20" customHeight="1">
       <c r="A29" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>124</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="20" customHeight="1">
@@ -2007,7 +2013,7 @@
         <v>125</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="20" customHeight="1">
@@ -2018,7 +2024,7 @@
         <v>126</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="20" customHeight="1">
@@ -2029,7 +2035,7 @@
         <v>127</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="20" customHeight="1">
@@ -2040,7 +2046,7 @@
         <v>128</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="20" customHeight="1">
@@ -2051,18 +2057,18 @@
         <v>129</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="20" customHeight="1">
       <c r="A35" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>130</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="20" customHeight="1">
@@ -2073,7 +2079,7 @@
         <v>131</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="37" spans="1:3" ht="20" customHeight="1">
@@ -2084,7 +2090,7 @@
         <v>132</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="38" spans="1:3" ht="20" customHeight="1">
@@ -2095,7 +2101,7 @@
         <v>133</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="20" customHeight="1">
@@ -2106,7 +2112,7 @@
         <v>134</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
     </row>
     <row r="40" spans="1:3" ht="20" customHeight="1">
@@ -2117,18 +2123,18 @@
         <v>135</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
     </row>
     <row r="41" spans="1:3" ht="20" customHeight="1">
       <c r="A41" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>136</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="42" spans="1:3" ht="20" customHeight="1">
@@ -2139,7 +2145,7 @@
         <v>137</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="43" spans="1:3" ht="20" customHeight="1">
@@ -2150,7 +2156,7 @@
         <v>138</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="20" customHeight="1">
@@ -2161,18 +2167,18 @@
         <v>139</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
     </row>
     <row r="45" spans="1:3" ht="20" customHeight="1">
       <c r="A45" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>140</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="46" spans="1:3" ht="20" customHeight="1">
@@ -2183,7 +2189,7 @@
         <v>141</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="47" spans="1:3" ht="20" customHeight="1">
@@ -2194,7 +2200,7 @@
         <v>142</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="48" spans="1:3" ht="20" customHeight="1">
@@ -2205,7 +2211,7 @@
         <v>143</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="20" customHeight="1">
@@ -2216,18 +2222,18 @@
         <v>144</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="50" spans="1:3" ht="20" customHeight="1">
       <c r="A50" s="1" t="s">
-        <v>93</v>
+        <v>31</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>145</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="51" spans="1:3" ht="20" customHeight="1">
@@ -2238,7 +2244,7 @@
         <v>146</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="52" spans="1:3" ht="20" customHeight="1">
@@ -2249,7 +2255,7 @@
         <v>147</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="53" spans="1:3" ht="20" customHeight="1">
@@ -2260,7 +2266,7 @@
         <v>148</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="54" spans="1:3" ht="20" customHeight="1">
@@ -2268,21 +2274,21 @@
         <v>93</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>206</v>
+        <v>221</v>
       </c>
     </row>
     <row r="55" spans="1:3" ht="20" customHeight="1">
       <c r="A55" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
     </row>
     <row r="56" spans="1:3" ht="20" customHeight="1">
@@ -2293,7 +2299,7 @@
         <v>150</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="57" spans="1:3" ht="20" customHeight="1">
@@ -2304,7 +2310,7 @@
         <v>151</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="58" spans="1:3" ht="20" customHeight="1">
@@ -2315,7 +2321,7 @@
         <v>152</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="59" spans="1:3" ht="20" customHeight="1">
@@ -2323,21 +2329,21 @@
         <v>94</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>135</v>
+        <v>153</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="60" spans="1:3" ht="20" customHeight="1">
       <c r="A60" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="61" spans="1:3" ht="20" customHeight="1">
@@ -2348,7 +2354,7 @@
         <v>154</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="62" spans="1:3" ht="20" customHeight="1">
@@ -2359,7 +2365,7 @@
         <v>155</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="63" spans="1:3" ht="20" customHeight="1">
@@ -2370,7 +2376,7 @@
         <v>156</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="64" spans="1:3" ht="20" customHeight="1">
@@ -2381,7 +2387,7 @@
         <v>157</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="65" spans="1:3" ht="20" customHeight="1">
@@ -2389,21 +2395,21 @@
         <v>95</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>135</v>
+        <v>158</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>206</v>
+        <v>231</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="20" customHeight="1">
       <c r="A66" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>158</v>
+        <v>136</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>230</v>
+        <v>208</v>
       </c>
     </row>
     <row r="67" spans="1:3" ht="20" customHeight="1">
@@ -2414,7 +2420,7 @@
         <v>159</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="68" spans="1:3" ht="20" customHeight="1">
@@ -2425,7 +2431,7 @@
         <v>160</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="69" spans="1:3" ht="20" customHeight="1">
@@ -2436,7 +2442,7 @@
         <v>161</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="70" spans="1:3" ht="20" customHeight="1">
@@ -2447,7 +2453,7 @@
         <v>162</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="71" spans="1:3" ht="20" customHeight="1">
@@ -2458,7 +2464,7 @@
         <v>163</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="72" spans="1:3" ht="20" customHeight="1">
@@ -2469,7 +2475,7 @@
         <v>164</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="73" spans="1:3" ht="20" customHeight="1">
@@ -2480,7 +2486,7 @@
         <v>165</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="74" spans="1:3" ht="20" customHeight="1">
@@ -2491,7 +2497,7 @@
         <v>166</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="75" spans="1:3" ht="20" customHeight="1">
@@ -2502,7 +2508,7 @@
         <v>167</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="76" spans="1:3" ht="20" customHeight="1">
@@ -2510,10 +2516,21 @@
         <v>96</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>135</v>
+        <v>168</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>206</v>
+        <v>241</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" ht="20" customHeight="1">
+      <c r="A77" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -2531,36 +2548,36 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="100" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Solución de envíos, fotos y clave
</commit_message>
<xml_diff>
--- a/SIG_MotMot_Validacion_Campo.xlsx
+++ b/SIG_MotMot_Validacion_Campo.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="260">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="254">
   <si>
     <t>type</t>
   </si>
@@ -42,12 +42,6 @@
     <t>select_one servicio</t>
   </si>
   <si>
-    <t>note</t>
-  </si>
-  <si>
-    <t>begin_repeat</t>
-  </si>
-  <si>
     <t>select_one tipo_punto</t>
   </si>
   <si>
@@ -87,9 +81,6 @@
     <t>image</t>
   </si>
   <si>
-    <t>end_repeat</t>
-  </si>
-  <si>
     <t>file</t>
   </si>
   <si>
@@ -99,12 +90,6 @@
     <t>servicio</t>
   </si>
   <si>
-    <t>nota_ayuda</t>
-  </si>
-  <si>
-    <t>puntos_ruta</t>
-  </si>
-  <si>
     <t>tipo_punto</t>
   </si>
   <si>
@@ -183,22 +168,16 @@
     <t>archivo_track</t>
   </si>
   <si>
-    <t>Nombre del evaluador</t>
-  </si>
-  <si>
-    <t>Servicio operativo a evaluar</t>
-  </si>
-  <si>
-    <t>💡 Use el botón "+" para agregar todos los puntos y riesgos que encuentre en el camino sin salir del formulario.</t>
-  </si>
-  <si>
-    <t>📍 Agregar Punto en la Ruta</t>
-  </si>
-  <si>
-    <t>Tipo de punto evaluado</t>
-  </si>
-  <si>
-    <t>Capturar ubicación GPS exacta (Registra Altitud/Desnivel)</t>
+    <t>1. Nombre del evaluador</t>
+  </si>
+  <si>
+    <t>2. Ruta a evaluar</t>
+  </si>
+  <si>
+    <t>3. ¿Qué vas a reportar aquí?</t>
+  </si>
+  <si>
+    <t>4. Capturar ubicación GPS exacta</t>
   </si>
   <si>
     <t>Instrucciones: ¿Qué camino tomar en esta bifurcación?</t>
@@ -213,64 +192,64 @@
     <t>Especifique otro tipo de peligro</t>
   </si>
   <si>
-    <t>Descripción específica del peligro en el entorno</t>
+    <t>Descripción específica del peligro</t>
   </si>
   <si>
     <t>Posibilidad de ocurrencia</t>
   </si>
   <si>
-    <t>Severidad de la consecuencia</t>
-  </si>
-  <si>
-    <t>Medida de control propuesta in situ (Evitar/Mitigar)</t>
-  </si>
-  <si>
-    <t>Logística de Evacuación y Apoyo</t>
+    <t>Severidad</t>
+  </si>
+  <si>
+    <t>Medida de control in situ (Evitar/Mitigar)</t>
+  </si>
+  <si>
+    <t>Punto de Evacuación / Rescate</t>
   </si>
   <si>
     <t>Viabilidad de acceso para rescate</t>
   </si>
   <si>
-    <t>Especifique otro método de acceso</t>
-  </si>
-  <si>
-    <t>Cobertura de telecomunicaciones celular</t>
-  </si>
-  <si>
-    <t>Especifique la red celular</t>
-  </si>
-  <si>
-    <t>Tiempo estimado de evacuación a centro médico</t>
-  </si>
-  <si>
-    <t>Especifique el tiempo exacto estimado</t>
-  </si>
-  <si>
-    <t>Punto de refugio, finca o contacto local adicional (Opcional)</t>
-  </si>
-  <si>
-    <t>Teléfono del refugio o contacto local (Opcional)</t>
-  </si>
-  <si>
-    <t>Interpretación y Confort Logístico</t>
+    <t>Especifique otro método</t>
+  </si>
+  <si>
+    <t>Cobertura celular</t>
+  </si>
+  <si>
+    <t>Especifique red celular</t>
+  </si>
+  <si>
+    <t>Tiempo estimado de evacuación</t>
+  </si>
+  <si>
+    <t>Especifique el tiempo exacto</t>
+  </si>
+  <si>
+    <t>Finca o contacto local (Opcional)</t>
+  </si>
+  <si>
+    <t>Teléfono del contacto (Opcional)</t>
+  </si>
+  <si>
+    <t>Punto de Confort / Interés</t>
   </si>
   <si>
     <t>Categoría del punto</t>
   </si>
   <si>
-    <t>Especifique otro punto de interés</t>
-  </si>
-  <si>
-    <t>Guion interpretativo / Información de valor a transmitir</t>
+    <t>Especifique otro</t>
+  </si>
+  <si>
+    <t>Guion interpretativo (Opcional)</t>
   </si>
   <si>
     <t>Observaciones logísticas</t>
   </si>
   <si>
-    <t>Evidencia fotográfica del lugar/punto (Opcional para Inicio/Fin, Recomendada para Bifurcaciones, Obligatoria para Riesgos/Evacuación)</t>
-  </si>
-  <si>
-    <t>Adjuntar archivo GPX/KML del track de la ruta (Al finalizar)</t>
+    <t>📸 Evidencia fotográfica del lugar</t>
+  </si>
+  <si>
+    <t>🗺️ Adjuntar archivo GPX/KML del track (Solo al llegar al final)</t>
   </si>
   <si>
     <t>yes</t>
@@ -315,6 +294,9 @@
     <t>selected(${cat_interes}, 'otro')</t>
   </si>
   <si>
+    <t>${tipo_punto} = 'fin'</t>
+  </si>
+  <si>
     <t>list_name</t>
   </si>
   <si>
@@ -678,31 +660,34 @@
     <t>Casi seguro</t>
   </si>
   <si>
-    <t>Insignificante (Sin lesiones)</t>
-  </si>
-  <si>
-    <t>Menor (Primeros auxilios básicos)</t>
-  </si>
-  <si>
-    <t>Moderada (Requiere atención médica)</t>
-  </si>
-  <si>
-    <t>Mayor (Evacuación inmediata)</t>
+    <t>Insignificante</t>
+  </si>
+  <si>
+    <t>Menor</t>
+  </si>
+  <si>
+    <t>Moderada</t>
+  </si>
+  <si>
+    <t>Mayor</t>
   </si>
   <si>
     <t>Catastrófica</t>
   </si>
   <si>
-    <t>Peatonal (Extracción en camilla)</t>
-  </si>
-  <si>
-    <t>Tracción animal (Mulas)</t>
+    <t>Peatonal</t>
+  </si>
+  <si>
+    <t>Tracción animal</t>
   </si>
   <si>
     <t>Vehicular 4x4</t>
   </si>
   <si>
-    <t>Acceso remoto crítico (Helitransportado)</t>
+    <t>Helitransportado</t>
+  </si>
+  <si>
+    <t>Otro</t>
   </si>
   <si>
     <t>Sin cobertura celular</t>
@@ -735,37 +720,34 @@
     <t>Un día o más</t>
   </si>
   <si>
-    <t>Otro</t>
-  </si>
-  <si>
-    <t>Zona de sombra natural / Descanso</t>
-  </si>
-  <si>
-    <t>Zona de relajación</t>
-  </si>
-  <si>
-    <t>Zona para acampar / Refugio</t>
+    <t>Descanso / Sombra</t>
+  </si>
+  <si>
+    <t>Relajación</t>
+  </si>
+  <si>
+    <t>Acampar / Refugio</t>
   </si>
   <si>
     <t>Punto hídrico</t>
   </si>
   <si>
-    <t>Servicios sanitarios</t>
-  </si>
-  <si>
-    <t>Zona de alimentación</t>
-  </si>
-  <si>
-    <t>Mirador panorámico</t>
-  </si>
-  <si>
-    <t>Interacción comunitaria</t>
-  </si>
-  <si>
-    <t>Observación de avifauna</t>
-  </si>
-  <si>
-    <t>Patrimonio arquitectónico</t>
+    <t>Baños</t>
+  </si>
+  <si>
+    <t>Alimentación</t>
+  </si>
+  <si>
+    <t>Mirador</t>
+  </si>
+  <si>
+    <t>Comunidad / Artesanos</t>
+  </si>
+  <si>
+    <t>Avifauna</t>
+  </si>
+  <si>
+    <t>Patrimonio</t>
   </si>
   <si>
     <t>form_title</t>
@@ -783,10 +765,10 @@
     <t>logo</t>
   </si>
   <si>
-    <t>Validación SIG ISO 21101 - Mot Mot Experiencias</t>
-  </si>
-  <si>
-    <t>sig_motmot_v7</t>
+    <t>Validación ISO 21101 - Mot Mot Experiencias</t>
+  </si>
+  <si>
+    <t>sig_motmot_v8_final</t>
   </si>
   <si>
     <t>Español</t>
@@ -1225,7 +1207,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="6" width="28.7109375" style="1" customWidth="1"/>
@@ -1256,16 +1238,16 @@
         <v>6</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -1273,13 +1255,13 @@
         <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -1287,10 +1269,13 @@
         <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -1298,10 +1283,13 @@
         <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>58</v>
+        <v>53</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -1309,13 +1297,16 @@
         <v>10</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>85</v>
+        <v>78</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -1323,13 +1314,13 @@
         <v>11</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>85</v>
+        <v>55</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -1337,391 +1328,355 @@
         <v>12</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>62</v>
+        <v>57</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>78</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="1" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>85</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>85</v>
+        <v>62</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>69</v>
+        <v>64</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>78</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="1" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F23" s="1" t="s">
-        <v>96</v>
+        <v>79</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>86</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>88</v>
+        <v>71</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="1" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>39</v>
+        <v>44</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C27" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D27" s="1" t="s">
         <v>78</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="1" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C28" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D28" s="1" t="s">
         <v>79</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F29" s="1" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D30" s="1" t="s">
-        <v>86</v>
+        <v>43</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="1" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C31" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E31" s="1" t="s">
         <v>82</v>
-      </c>
-      <c r="D31" s="1" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5">
-      <c r="A33" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="E33" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5">
-      <c r="A34" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5">
-      <c r="A35" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D35" s="1" t="s">
-        <v>86</v>
+        <v>49</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -1739,7 +1694,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="30" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -1750,838 +1705,838 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>123</v>
+        <v>117</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
     </row>
     <row r="27" spans="1:3">
       <c r="A27" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="28" spans="1:3">
       <c r="A28" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
     </row>
     <row r="29" spans="1:3">
       <c r="A29" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
     </row>
     <row r="30" spans="1:3">
       <c r="A30" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
     <row r="33" spans="1:3">
       <c r="A33" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
     </row>
     <row r="34" spans="1:3">
       <c r="A34" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
     </row>
     <row r="35" spans="1:3">
       <c r="A35" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="36" spans="1:3">
       <c r="A36" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
     </row>
     <row r="39" spans="1:3">
       <c r="A39" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="41" spans="1:3">
       <c r="A41" s="1" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
     </row>
     <row r="42" spans="1:3">
       <c r="A42" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" s="1" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" s="1" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" s="1" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="53" spans="1:3">
       <c r="A53" s="1" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" s="1" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
     </row>
     <row r="55" spans="1:3">
       <c r="A55" s="1" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" s="1" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
     </row>
     <row r="57" spans="1:3">
       <c r="A57" s="1" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
     </row>
     <row r="58" spans="1:3">
       <c r="A58" s="1" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
     </row>
     <row r="59" spans="1:3">
       <c r="A59" s="1" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="60" spans="1:3">
       <c r="A60" s="1" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" s="1" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>234</v>
+        <v>229</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" s="1" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>235</v>
+        <v>230</v>
       </c>
     </row>
     <row r="63" spans="1:3">
       <c r="A63" s="1" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>236</v>
+        <v>231</v>
       </c>
     </row>
     <row r="64" spans="1:3">
       <c r="A64" s="1" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
     </row>
     <row r="65" spans="1:3">
       <c r="A65" s="1" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="66" spans="1:3">
       <c r="A66" s="1" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>239</v>
+        <v>223</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
     </row>
     <row r="68" spans="1:3">
       <c r="A68" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
     </row>
     <row r="70" spans="1:3">
       <c r="A70" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
     </row>
     <row r="72" spans="1:3">
       <c r="A72" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
     </row>
     <row r="73" spans="1:3">
       <c r="A73" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
     </row>
     <row r="76" spans="1:3">
       <c r="A76" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
     </row>
     <row r="77" spans="1:3">
       <c r="A77" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>239</v>
+        <v>223</v>
       </c>
     </row>
   </sheetData>
@@ -2599,36 +2554,36 @@
   <sheetData>
     <row r="1" spans="1:5" ht="30" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
     </row>
   </sheetData>

</xml_diff>